<commit_message>
Fix department naming and regenerate processed data
</commit_message>
<xml_diff>
--- a/data/processed/encoded_dataset.xlsx
+++ b/data/processed/encoded_dataset.xlsx
@@ -546,7 +546,7 @@
         <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E2" t="n">
         <v>23</v>
@@ -676,7 +676,7 @@
         <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E4" t="n">
         <v>12</v>
@@ -806,7 +806,7 @@
         <v>5</v>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E6" t="n">
         <v>11</v>
@@ -936,7 +936,7 @@
         <v>5</v>
       </c>
       <c r="D8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E8" t="n">
         <v>12</v>
@@ -1001,7 +1001,7 @@
         <v>4</v>
       </c>
       <c r="D9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E9" t="n">
         <v>7</v>
@@ -1066,7 +1066,7 @@
         <v>4</v>
       </c>
       <c r="D10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E10" t="n">
         <v>25</v>
@@ -1131,7 +1131,7 @@
         <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E11" t="n">
         <v>5</v>
@@ -1196,7 +1196,7 @@
         <v>5</v>
       </c>
       <c r="D12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E12" t="n">
         <v>7</v>
@@ -1261,7 +1261,7 @@
         <v>2</v>
       </c>
       <c r="D13" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E13" t="n">
         <v>5</v>
@@ -1651,7 +1651,7 @@
         <v>4</v>
       </c>
       <c r="D19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E19" t="n">
         <v>26</v>
@@ -1716,7 +1716,7 @@
         <v>4</v>
       </c>
       <c r="D20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E20" t="n">
         <v>5</v>
@@ -1781,7 +1781,7 @@
         <v>4</v>
       </c>
       <c r="D21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E21" t="n">
         <v>15</v>
@@ -1846,7 +1846,7 @@
         <v>4</v>
       </c>
       <c r="D22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E22" t="n">
         <v>26</v>
@@ -1911,7 +1911,7 @@
         <v>2</v>
       </c>
       <c r="D23" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E23" t="n">
         <v>8</v>
@@ -1976,7 +1976,7 @@
         <v>4</v>
       </c>
       <c r="D24" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E24" t="n">
         <v>7</v>
@@ -2041,7 +2041,7 @@
         <v>5</v>
       </c>
       <c r="D25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
@@ -2171,7 +2171,7 @@
         <v>3</v>
       </c>
       <c r="D27" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E27" t="n">
         <v>25</v>
@@ -2236,7 +2236,7 @@
         <v>3</v>
       </c>
       <c r="D28" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E28" t="n">
         <v>14</v>
@@ -2301,7 +2301,7 @@
         <v>4</v>
       </c>
       <c r="D29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E29" t="n">
         <v>2</v>
@@ -2366,7 +2366,7 @@
         <v>4</v>
       </c>
       <c r="D30" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E30" t="n">
         <v>21</v>
@@ -2431,7 +2431,7 @@
         <v>4</v>
       </c>
       <c r="D31" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E31" t="n">
         <v>16</v>
@@ -2561,7 +2561,7 @@
         <v>3</v>
       </c>
       <c r="D33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E33" t="n">
         <v>9</v>
@@ -2691,7 +2691,7 @@
         <v>2</v>
       </c>
       <c r="D35" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E35" t="n">
         <v>14</v>
@@ -2756,7 +2756,7 @@
         <v>4</v>
       </c>
       <c r="D36" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E36" t="n">
         <v>14</v>
@@ -2821,7 +2821,7 @@
         <v>2</v>
       </c>
       <c r="D37" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E37" t="n">
         <v>7</v>
@@ -2886,7 +2886,7 @@
         <v>3</v>
       </c>
       <c r="D38" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E38" t="n">
         <v>21</v>
@@ -2951,7 +2951,7 @@
         <v>4</v>
       </c>
       <c r="D39" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E39" t="n">
         <v>7</v>
@@ -3081,7 +3081,7 @@
         <v>5</v>
       </c>
       <c r="D41" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E41" t="n">
         <v>14</v>
@@ -3211,7 +3211,7 @@
         <v>2</v>
       </c>
       <c r="D43" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E43" t="n">
         <v>16</v>
@@ -3276,7 +3276,7 @@
         <v>4</v>
       </c>
       <c r="D44" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E44" t="n">
         <v>7</v>
@@ -3341,7 +3341,7 @@
         <v>5</v>
       </c>
       <c r="D45" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E45" t="n">
         <v>8</v>
@@ -3406,7 +3406,7 @@
         <v>4</v>
       </c>
       <c r="D46" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E46" t="n">
         <v>14</v>
@@ -3471,7 +3471,7 @@
         <v>4</v>
       </c>
       <c r="D47" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E47" t="n">
         <v>15</v>
@@ -3601,7 +3601,7 @@
         <v>5</v>
       </c>
       <c r="D49" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E49" t="n">
         <v>12</v>
@@ -3666,7 +3666,7 @@
         <v>4</v>
       </c>
       <c r="D50" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E50" t="n">
         <v>15</v>
@@ -3796,7 +3796,7 @@
         <v>4</v>
       </c>
       <c r="D52" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E52" t="n">
         <v>8</v>
@@ -3991,7 +3991,7 @@
         <v>3</v>
       </c>
       <c r="D55" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E55" t="n">
         <v>5</v>
@@ -4056,7 +4056,7 @@
         <v>2</v>
       </c>
       <c r="D56" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E56" t="n">
         <v>11</v>
@@ -4121,7 +4121,7 @@
         <v>3</v>
       </c>
       <c r="D57" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E57" t="n">
         <v>25</v>
@@ -4186,7 +4186,7 @@
         <v>2</v>
       </c>
       <c r="D58" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E58" t="n">
         <v>26</v>
@@ -4316,7 +4316,7 @@
         <v>3</v>
       </c>
       <c r="D60" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E60" t="n">
         <v>2</v>
@@ -4446,7 +4446,7 @@
         <v>2</v>
       </c>
       <c r="D62" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E62" t="n">
         <v>20</v>
@@ -4511,7 +4511,7 @@
         <v>3</v>
       </c>
       <c r="D63" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E63" t="n">
         <v>5</v>
@@ -4576,7 +4576,7 @@
         <v>2</v>
       </c>
       <c r="D64" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E64" t="n">
         <v>8</v>
@@ -4641,7 +4641,7 @@
         <v>4</v>
       </c>
       <c r="D65" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E65" t="n">
         <v>26</v>
@@ -4706,7 +4706,7 @@
         <v>2</v>
       </c>
       <c r="D66" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E66" t="n">
         <v>8</v>
@@ -4771,7 +4771,7 @@
         <v>3</v>
       </c>
       <c r="D67" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E67" t="n">
         <v>26</v>
@@ -4901,7 +4901,7 @@
         <v>2</v>
       </c>
       <c r="D69" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E69" t="n">
         <v>20</v>
@@ -4966,7 +4966,7 @@
         <v>5</v>
       </c>
       <c r="D70" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E70" t="n">
         <v>14</v>
@@ -5031,7 +5031,7 @@
         <v>5</v>
       </c>
       <c r="D71" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E71" t="n">
         <v>11</v>
@@ -5096,7 +5096,7 @@
         <v>3</v>
       </c>
       <c r="D72" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E72" t="n">
         <v>9</v>
@@ -5161,7 +5161,7 @@
         <v>2</v>
       </c>
       <c r="D73" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E73" t="n">
         <v>27</v>
@@ -5226,7 +5226,7 @@
         <v>3</v>
       </c>
       <c r="D74" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E74" t="n">
         <v>8</v>
@@ -5291,7 +5291,7 @@
         <v>3</v>
       </c>
       <c r="D75" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E75" t="n">
         <v>11</v>
@@ -5356,7 +5356,7 @@
         <v>4</v>
       </c>
       <c r="D76" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E76" t="n">
         <v>16</v>
@@ -5421,7 +5421,7 @@
         <v>2</v>
       </c>
       <c r="D77" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E77" t="n">
         <v>25</v>
@@ -5486,7 +5486,7 @@
         <v>3</v>
       </c>
       <c r="D78" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E78" t="n">
         <v>23</v>
@@ -5551,7 +5551,7 @@
         <v>3</v>
       </c>
       <c r="D79" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E79" t="n">
         <v>2</v>
@@ -5616,7 +5616,7 @@
         <v>3</v>
       </c>
       <c r="D80" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E80" t="n">
         <v>16</v>
@@ -5746,7 +5746,7 @@
         <v>4</v>
       </c>
       <c r="D82" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E82" t="n">
         <v>8</v>
@@ -5811,7 +5811,7 @@
         <v>3</v>
       </c>
       <c r="D83" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E83" t="n">
         <v>14</v>
@@ -5941,7 +5941,7 @@
         <v>2</v>
       </c>
       <c r="D85" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E85" t="n">
         <v>23</v>
@@ -6006,7 +6006,7 @@
         <v>3</v>
       </c>
       <c r="D86" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E86" t="n">
         <v>11</v>
@@ -6071,7 +6071,7 @@
         <v>5</v>
       </c>
       <c r="D87" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E87" t="n">
         <v>25</v>
@@ -6136,7 +6136,7 @@
         <v>3</v>
       </c>
       <c r="D88" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E88" t="n">
         <v>0</v>
@@ -6201,7 +6201,7 @@
         <v>4</v>
       </c>
       <c r="D89" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E89" t="n">
         <v>27</v>
@@ -6396,7 +6396,7 @@
         <v>3</v>
       </c>
       <c r="D92" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E92" t="n">
         <v>25</v>
@@ -6526,7 +6526,7 @@
         <v>2</v>
       </c>
       <c r="D94" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E94" t="n">
         <v>15</v>
@@ -6656,7 +6656,7 @@
         <v>2</v>
       </c>
       <c r="D96" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E96" t="n">
         <v>2</v>
@@ -6721,7 +6721,7 @@
         <v>2</v>
       </c>
       <c r="D97" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E97" t="n">
         <v>8</v>
@@ -6786,7 +6786,7 @@
         <v>3</v>
       </c>
       <c r="D98" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E98" t="n">
         <v>6</v>
@@ -6851,7 +6851,7 @@
         <v>2</v>
       </c>
       <c r="D99" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E99" t="n">
         <v>8</v>
@@ -6916,7 +6916,7 @@
         <v>4</v>
       </c>
       <c r="D100" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E100" t="n">
         <v>25</v>
@@ -6981,7 +6981,7 @@
         <v>2</v>
       </c>
       <c r="D101" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E101" t="n">
         <v>8</v>
@@ -7046,7 +7046,7 @@
         <v>3</v>
       </c>
       <c r="D102" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E102" t="n">
         <v>25</v>
@@ -7176,7 +7176,7 @@
         <v>3</v>
       </c>
       <c r="D104" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E104" t="n">
         <v>25</v>
@@ -7241,7 +7241,7 @@
         <v>4</v>
       </c>
       <c r="D105" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E105" t="n">
         <v>25</v>
@@ -7306,7 +7306,7 @@
         <v>2</v>
       </c>
       <c r="D106" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E106" t="n">
         <v>12</v>
@@ -7371,7 +7371,7 @@
         <v>2</v>
       </c>
       <c r="D107" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E107" t="n">
         <v>11</v>
@@ -7436,7 +7436,7 @@
         <v>2</v>
       </c>
       <c r="D108" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E108" t="n">
         <v>25</v>
@@ -7501,7 +7501,7 @@
         <v>5</v>
       </c>
       <c r="D109" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E109" t="n">
         <v>23</v>
@@ -7566,7 +7566,7 @@
         <v>3</v>
       </c>
       <c r="D110" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E110" t="n">
         <v>6</v>
@@ -7631,7 +7631,7 @@
         <v>3</v>
       </c>
       <c r="D111" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E111" t="n">
         <v>0</v>
@@ -7696,7 +7696,7 @@
         <v>4</v>
       </c>
       <c r="D112" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E112" t="n">
         <v>0</v>
@@ -7826,7 +7826,7 @@
         <v>5</v>
       </c>
       <c r="D114" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E114" t="n">
         <v>0</v>
@@ -7956,7 +7956,7 @@
         <v>2</v>
       </c>
       <c r="D116" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E116" t="n">
         <v>19</v>
@@ -8086,7 +8086,7 @@
         <v>3</v>
       </c>
       <c r="D118" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E118" t="n">
         <v>15</v>
@@ -8151,7 +8151,7 @@
         <v>5</v>
       </c>
       <c r="D119" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E119" t="n">
         <v>27</v>
@@ -8216,7 +8216,7 @@
         <v>3</v>
       </c>
       <c r="D120" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E120" t="n">
         <v>25</v>
@@ -8346,7 +8346,7 @@
         <v>3</v>
       </c>
       <c r="D122" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E122" t="n">
         <v>0</v>
@@ -8411,7 +8411,7 @@
         <v>2</v>
       </c>
       <c r="D123" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E123" t="n">
         <v>5</v>
@@ -8606,7 +8606,7 @@
         <v>2</v>
       </c>
       <c r="D126" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E126" t="n">
         <v>5</v>
@@ -8736,7 +8736,7 @@
         <v>2</v>
       </c>
       <c r="D128" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E128" t="n">
         <v>20</v>
@@ -8801,7 +8801,7 @@
         <v>3</v>
       </c>
       <c r="D129" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E129" t="n">
         <v>7</v>
@@ -8866,7 +8866,7 @@
         <v>4</v>
       </c>
       <c r="D130" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E130" t="n">
         <v>7</v>
@@ -8931,7 +8931,7 @@
         <v>5</v>
       </c>
       <c r="D131" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E131" t="n">
         <v>10</v>
@@ -8996,7 +8996,7 @@
         <v>2</v>
       </c>
       <c r="D132" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E132" t="n">
         <v>5</v>
@@ -9126,7 +9126,7 @@
         <v>2</v>
       </c>
       <c r="D134" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E134" t="n">
         <v>26</v>
@@ -9191,7 +9191,7 @@
         <v>3</v>
       </c>
       <c r="D135" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E135" t="n">
         <v>16</v>
@@ -9321,7 +9321,7 @@
         <v>2</v>
       </c>
       <c r="D137" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E137" t="n">
         <v>23</v>
@@ -9451,7 +9451,7 @@
         <v>3</v>
       </c>
       <c r="D139" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E139" t="n">
         <v>11</v>
@@ -9516,7 +9516,7 @@
         <v>3</v>
       </c>
       <c r="D140" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E140" t="n">
         <v>25</v>
@@ -9581,7 +9581,7 @@
         <v>5</v>
       </c>
       <c r="D141" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E141" t="n">
         <v>9</v>
@@ -9646,7 +9646,7 @@
         <v>4</v>
       </c>
       <c r="D142" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E142" t="n">
         <v>21</v>
@@ -9776,7 +9776,7 @@
         <v>4</v>
       </c>
       <c r="D144" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E144" t="n">
         <v>15</v>
@@ -9841,7 +9841,7 @@
         <v>2</v>
       </c>
       <c r="D145" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E145" t="n">
         <v>6</v>
@@ -9906,7 +9906,7 @@
         <v>3</v>
       </c>
       <c r="D146" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E146" t="n">
         <v>16</v>
@@ -9971,7 +9971,7 @@
         <v>5</v>
       </c>
       <c r="D147" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E147" t="n">
         <v>15</v>
@@ -10036,7 +10036,7 @@
         <v>2</v>
       </c>
       <c r="D148" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E148" t="n">
         <v>8</v>
@@ -10101,7 +10101,7 @@
         <v>3</v>
       </c>
       <c r="D149" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E149" t="n">
         <v>25</v>
@@ -10231,7 +10231,7 @@
         <v>2</v>
       </c>
       <c r="D151" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E151" t="n">
         <v>14</v>
@@ -10296,7 +10296,7 @@
         <v>3</v>
       </c>
       <c r="D152" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E152" t="n">
         <v>0</v>
@@ -10361,7 +10361,7 @@
         <v>3</v>
       </c>
       <c r="D153" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E153" t="n">
         <v>8</v>
@@ -10426,7 +10426,7 @@
         <v>3</v>
       </c>
       <c r="D154" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E154" t="n">
         <v>8</v>
@@ -10491,7 +10491,7 @@
         <v>3</v>
       </c>
       <c r="D155" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E155" t="n">
         <v>10</v>
@@ -10556,7 +10556,7 @@
         <v>2</v>
       </c>
       <c r="D156" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E156" t="n">
         <v>16</v>
@@ -10621,7 +10621,7 @@
         <v>5</v>
       </c>
       <c r="D157" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E157" t="n">
         <v>19</v>
@@ -10751,7 +10751,7 @@
         <v>2</v>
       </c>
       <c r="D159" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E159" t="n">
         <v>26</v>
@@ -10946,7 +10946,7 @@
         <v>3</v>
       </c>
       <c r="D162" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E162" t="n">
         <v>10</v>
@@ -11011,7 +11011,7 @@
         <v>2</v>
       </c>
       <c r="D163" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E163" t="n">
         <v>26</v>
@@ -11076,7 +11076,7 @@
         <v>3</v>
       </c>
       <c r="D164" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E164" t="n">
         <v>25</v>
@@ -11141,7 +11141,7 @@
         <v>4</v>
       </c>
       <c r="D165" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E165" t="n">
         <v>0</v>
@@ -11206,7 +11206,7 @@
         <v>2</v>
       </c>
       <c r="D166" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E166" t="n">
         <v>0</v>
@@ -11336,7 +11336,7 @@
         <v>2</v>
       </c>
       <c r="D168" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E168" t="n">
         <v>25</v>
@@ -11401,7 +11401,7 @@
         <v>4</v>
       </c>
       <c r="D169" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E169" t="n">
         <v>7</v>
@@ -11531,7 +11531,7 @@
         <v>3</v>
       </c>
       <c r="D171" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E171" t="n">
         <v>5</v>
@@ -11596,7 +11596,7 @@
         <v>5</v>
       </c>
       <c r="D172" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E172" t="n">
         <v>23</v>
@@ -11661,7 +11661,7 @@
         <v>2</v>
       </c>
       <c r="D173" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E173" t="n">
         <v>11</v>
@@ -11856,7 +11856,7 @@
         <v>2</v>
       </c>
       <c r="D176" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E176" t="n">
         <v>23</v>
@@ -11921,7 +11921,7 @@
         <v>4</v>
       </c>
       <c r="D177" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E177" t="n">
         <v>14</v>
@@ -11986,7 +11986,7 @@
         <v>2</v>
       </c>
       <c r="D178" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E178" t="n">
         <v>16</v>
@@ -12116,7 +12116,7 @@
         <v>2</v>
       </c>
       <c r="D180" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E180" t="n">
         <v>0</v>
@@ -12181,7 +12181,7 @@
         <v>2</v>
       </c>
       <c r="D181" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E181" t="n">
         <v>2</v>
@@ -12246,7 +12246,7 @@
         <v>4</v>
       </c>
       <c r="D182" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E182" t="n">
         <v>8</v>
@@ -12311,7 +12311,7 @@
         <v>3</v>
       </c>
       <c r="D183" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E183" t="n">
         <v>15</v>
@@ -12376,7 +12376,7 @@
         <v>5</v>
       </c>
       <c r="D184" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E184" t="n">
         <v>8</v>
@@ -12441,7 +12441,7 @@
         <v>2</v>
       </c>
       <c r="D185" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E185" t="n">
         <v>14</v>
@@ -12506,7 +12506,7 @@
         <v>5</v>
       </c>
       <c r="D186" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E186" t="n">
         <v>5</v>
@@ -12571,7 +12571,7 @@
         <v>5</v>
       </c>
       <c r="D187" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E187" t="n">
         <v>16</v>
@@ -12636,7 +12636,7 @@
         <v>3</v>
       </c>
       <c r="D188" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E188" t="n">
         <v>0</v>
@@ -12701,7 +12701,7 @@
         <v>4</v>
       </c>
       <c r="D189" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E189" t="n">
         <v>10</v>
@@ -12766,7 +12766,7 @@
         <v>5</v>
       </c>
       <c r="D190" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E190" t="n">
         <v>16</v>
@@ -13026,7 +13026,7 @@
         <v>5</v>
       </c>
       <c r="D194" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E194" t="n">
         <v>19</v>
@@ -13091,7 +13091,7 @@
         <v>2</v>
       </c>
       <c r="D195" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E195" t="n">
         <v>20</v>
@@ -13156,7 +13156,7 @@
         <v>3</v>
       </c>
       <c r="D196" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E196" t="n">
         <v>14</v>
@@ -13221,7 +13221,7 @@
         <v>2</v>
       </c>
       <c r="D197" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E197" t="n">
         <v>25</v>
@@ -13286,7 +13286,7 @@
         <v>5</v>
       </c>
       <c r="D198" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E198" t="n">
         <v>8</v>
@@ -13351,7 +13351,7 @@
         <v>3</v>
       </c>
       <c r="D199" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E199" t="n">
         <v>19</v>
@@ -13416,7 +13416,7 @@
         <v>3</v>
       </c>
       <c r="D200" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E200" t="n">
         <v>7</v>
@@ -13546,7 +13546,7 @@
         <v>4</v>
       </c>
       <c r="D202" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E202" t="n">
         <v>8</v>
@@ -13936,7 +13936,7 @@
         <v>5</v>
       </c>
       <c r="D208" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E208" t="n">
         <v>18</v>

</xml_diff>